<commit_message>
pdf of the presentation
</commit_message>
<xml_diff>
--- a/RVHP.xlsx
+++ b/RVHP.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micha\Documents\models\models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8635566D-B93B-4B72-BCB0-2A0499C95593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C078126-98D8-4945-9926-CEC34AC84360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{7A1D45B4-DF5B-42E3-9D70-4CD0D41444C9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="2" xr2:uid="{7A1D45B4-DF5B-42E3-9D70-4CD0D41444C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
     <sheet name="brilaroxazine" sheetId="2" r:id="rId2"/>
+    <sheet name="Trial" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="50">
   <si>
     <t>Price</t>
   </si>
@@ -164,6 +165,18 @@
   </si>
   <si>
     <t>Cash. Val</t>
+  </si>
+  <si>
+    <t>NCT05184335</t>
+  </si>
+  <si>
+    <t>The total duration of the study is 56 weeks (28 days/4 weeks DB treatment and 52-weeks OL treatment).</t>
+  </si>
+  <si>
+    <t>Goal</t>
+  </si>
+  <si>
+    <t>ID</t>
   </si>
 </sst>
 </file>
@@ -173,7 +186,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -199,6 +212,11 @@
       <family val="2"/>
       <charset val="238"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF171716"/>
+      <name val="Roboto"/>
     </font>
     <font>
       <b/>
@@ -240,9 +258,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color rgb="FF1B1B1B"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
       <b/>
-      <u/>
-      <sz val="12"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -378,7 +400,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -394,17 +416,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -427,16 +452,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>96493</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>24020</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>394666</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>98563</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>154075</xdr:colOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>452249</xdr:colOff>
       <xdr:row>29</xdr:row>
-      <xdr:rowOff>151511</xdr:rowOff>
+      <xdr:rowOff>27272</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -459,8 +484,52 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11410536" y="421585"/>
+          <a:off x="12321623" y="297346"/>
           <a:ext cx="3122148" cy="5478056"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>298173</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>74543</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>509317</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>120628</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5A1B0759-1823-4AB3-88EB-4FBE3FFF4F9B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7321825" y="2451652"/>
+          <a:ext cx="5114449" cy="3027824"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -778,16 +847,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
     </row>
     <row r="2" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
-      <c r="J2" s="22"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
     </row>
     <row r="3" spans="3:16" x14ac:dyDescent="0.25">
       <c r="C3" s="5" t="s">
@@ -800,10 +869,10 @@
         <v>9</v>
       </c>
       <c r="F3" s="7"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="23"/>
       <c r="L3" t="s">
         <v>0</v>
       </c>
@@ -815,7 +884,7 @@
       </c>
     </row>
     <row r="4" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="16" t="s">
         <v>11</v>
       </c>
       <c r="D4" t="s">
@@ -824,11 +893,11 @@
       <c r="E4" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="23"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
       <c r="L4" t="s">
         <v>1</v>
       </c>
@@ -845,10 +914,10 @@
         <v>13</v>
       </c>
       <c r="F5" s="8"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="23"/>
+      <c r="J5" s="23"/>
       <c r="L5" t="s">
         <v>2</v>
       </c>
@@ -866,10 +935,10 @@
         <v>14</v>
       </c>
       <c r="F6" s="8"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="23"/>
       <c r="L6" t="s">
         <v>3</v>
       </c>
@@ -886,10 +955,10 @@
         <v>10</v>
       </c>
       <c r="F7" s="8"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
       <c r="L7" t="s">
         <v>4</v>
       </c>
@@ -905,10 +974,10 @@
         <v>42</v>
       </c>
       <c r="F8" s="8"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
-      <c r="I8" s="22"/>
-      <c r="J8" s="22"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="23"/>
       <c r="L8" t="s">
         <v>5</v>
       </c>
@@ -923,10 +992,10 @@
     <row r="9" spans="3:16" x14ac:dyDescent="0.25">
       <c r="C9" s="9"/>
       <c r="F9" s="8"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="22"/>
-      <c r="J9" s="22"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
+      <c r="J9" s="23"/>
       <c r="N9" s="3" t="s">
         <v>6</v>
       </c>
@@ -936,14 +1005,14 @@
       <c r="D10" s="11"/>
       <c r="E10" s="11"/>
       <c r="F10" s="12"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="22"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="23"/>
       <c r="L10" t="s">
         <v>45</v>
       </c>
-      <c r="M10" s="13">
+      <c r="M10" s="14">
         <f>+M6/M4</f>
         <v>0.18456375838926173</v>
       </c>
@@ -952,18 +1021,18 @@
       </c>
     </row>
     <row r="11" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="G11" s="22"/>
-      <c r="H11" s="22"/>
-      <c r="I11" s="22"/>
-      <c r="J11" s="22"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+      <c r="J11" s="23"/>
       <c r="O11" s="2"/>
       <c r="P11" s="3"/>
     </row>
     <row r="12" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="G12" s="22"/>
-      <c r="H12" s="22"/>
-      <c r="I12" s="22"/>
-      <c r="J12" s="22"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
+      <c r="J12" s="23"/>
       <c r="O12" s="2"/>
       <c r="P12" s="3"/>
     </row>
@@ -998,395 +1067,430 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
     </row>
     <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="16"/>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
     </row>
     <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="16"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="20" t="s">
+      <c r="A3" s="18"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
     </row>
     <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="16"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="20" t="s">
+      <c r="A4" s="18"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="16"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="16"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="18"/>
+      <c r="J4" s="18"/>
     </row>
     <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="16"/>
-      <c r="B5" s="16"/>
-      <c r="C5" s="20" t="s">
+      <c r="A5" s="18"/>
+      <c r="B5" s="18"/>
+      <c r="C5" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="16"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="18"/>
+      <c r="J5" s="18"/>
     </row>
     <row r="6" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="16"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="20" t="s">
+      <c r="A6" s="18"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="18">
         <v>1</v>
       </c>
-      <c r="E6" s="16" t="s">
+      <c r="E6" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="16"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
     </row>
     <row r="7" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="16"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="20" t="s">
+      <c r="A7" s="18"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="D7" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="16"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
     </row>
     <row r="8" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="16"/>
-      <c r="B8" s="16"/>
-      <c r="C8" s="20" t="s">
+      <c r="A8" s="18"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-      <c r="I8" s="16"/>
-      <c r="J8" s="16"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="18"/>
     </row>
     <row r="9" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="16"/>
-      <c r="B9" s="16"/>
-      <c r="C9" s="20" t="s">
+      <c r="A9" s="18"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="16"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="18"/>
+      <c r="J9" s="18"/>
     </row>
     <row r="10" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="16"/>
-      <c r="B10" s="16"/>
-      <c r="C10" s="20" t="s">
+      <c r="A10" s="18"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="18">
         <v>450</v>
       </c>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="16"/>
-      <c r="I10" s="16"/>
-      <c r="J10" s="16"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="18"/>
     </row>
     <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="16"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="20" t="s">
+      <c r="A11" s="18"/>
+      <c r="B11" s="18"/>
+      <c r="C11" s="22" t="s">
         <v>24</v>
       </c>
       <c r="D11" t="s">
         <v>31</v>
       </c>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="16"/>
-      <c r="I11" s="16"/>
-      <c r="J11" s="16"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="18"/>
+      <c r="J11" s="18"/>
     </row>
     <row r="12" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="20"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="16"/>
+      <c r="A12" s="18"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="22"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="18"/>
     </row>
     <row r="13" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
-      <c r="B13" s="16"/>
+      <c r="A13" s="18"/>
+      <c r="B13" s="18"/>
       <c r="C13" t="s">
         <v>33</v>
       </c>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
-      <c r="I13" s="16"/>
-      <c r="J13" s="16"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="18"/>
+      <c r="J13" s="18"/>
     </row>
     <row r="14" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="16"/>
-      <c r="B14" s="16"/>
+      <c r="A14" s="18"/>
+      <c r="B14" s="18"/>
       <c r="C14" t="s">
         <v>34</v>
       </c>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
-      <c r="I14" s="16"/>
-      <c r="J14" s="16"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="18"/>
+      <c r="J14" s="18"/>
     </row>
     <row r="15" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="16"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="19" t="s">
+      <c r="A15" s="18"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
-      <c r="I15" s="16"/>
-      <c r="J15" s="16"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="18"/>
+      <c r="J15" s="18"/>
     </row>
     <row r="16" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="16"/>
-      <c r="B16" s="16"/>
+      <c r="A16" s="18"/>
+      <c r="B16" s="18"/>
       <c r="C16" t="s">
         <v>36</v>
       </c>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="16"/>
-      <c r="I16" s="16"/>
-      <c r="J16" s="16"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="18"/>
+      <c r="J16" s="18"/>
     </row>
     <row r="17" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="16"/>
-      <c r="B17" s="16"/>
+      <c r="A17" s="18"/>
+      <c r="B17" s="18"/>
       <c r="C17" t="s">
         <v>37</v>
       </c>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="16"/>
-      <c r="I17" s="16"/>
-      <c r="J17" s="16"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="18"/>
+      <c r="J17" s="18"/>
     </row>
     <row r="18" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="16"/>
-      <c r="B18" s="16"/>
+      <c r="A18" s="18"/>
+      <c r="B18" s="18"/>
       <c r="C18" t="s">
         <v>38</v>
       </c>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
-      <c r="I18" s="16"/>
-      <c r="J18" s="16"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="18"/>
     </row>
     <row r="19" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="16"/>
-      <c r="B19" s="16"/>
+      <c r="A19" s="18"/>
+      <c r="B19" s="18"/>
       <c r="C19" t="s">
         <v>39</v>
       </c>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="16"/>
-      <c r="H19" s="16"/>
-      <c r="I19" s="16"/>
-      <c r="J19" s="16"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="18"/>
+      <c r="J19" s="18"/>
     </row>
     <row r="20" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="16"/>
-      <c r="B20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="16"/>
-      <c r="H20" s="16"/>
-      <c r="I20" s="16"/>
-      <c r="J20" s="16"/>
+      <c r="A20" s="18"/>
+      <c r="B20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
+      <c r="J20" s="18"/>
     </row>
     <row r="21" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="16"/>
-      <c r="B21" s="16"/>
-      <c r="C21" s="18"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="16"/>
-      <c r="H21" s="16"/>
-      <c r="I21" s="16"/>
-      <c r="J21" s="16"/>
+      <c r="A21" s="18"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="20"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="18"/>
+      <c r="H21" s="18"/>
+      <c r="I21" s="18"/>
+      <c r="J21" s="18"/>
     </row>
     <row r="22" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="16"/>
-      <c r="B22" s="16"/>
-      <c r="C22" s="21" t="s">
+      <c r="A22" s="18"/>
+      <c r="B22" s="18"/>
+      <c r="C22" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="16"/>
-      <c r="G22" s="16"/>
-      <c r="H22" s="16"/>
-      <c r="I22" s="16"/>
-      <c r="J22" s="16"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="18"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="18"/>
+      <c r="J22" s="18"/>
     </row>
     <row r="23" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="16"/>
-      <c r="B23" s="16"/>
-      <c r="C23" s="16" t="s">
+      <c r="A23" s="18"/>
+      <c r="B23" s="18"/>
+      <c r="C23" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="16"/>
-      <c r="G23" s="16"/>
-      <c r="H23" s="16"/>
-      <c r="I23" s="16"/>
-      <c r="J23" s="16"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="18"/>
+      <c r="G23" s="18"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="18"/>
+      <c r="J23" s="18"/>
     </row>
     <row r="24" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="16"/>
-      <c r="B24" s="16"/>
-      <c r="C24" s="16"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="16"/>
-      <c r="G24" s="16"/>
-      <c r="H24" s="16"/>
-      <c r="I24" s="16"/>
-      <c r="J24" s="16"/>
+      <c r="A24" s="18"/>
+      <c r="B24" s="18"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="18"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="18"/>
+      <c r="I24" s="18"/>
+      <c r="J24" s="18"/>
     </row>
     <row r="25" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="16"/>
-      <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="16"/>
-      <c r="H25" s="16"/>
-      <c r="I25" s="16"/>
-      <c r="J25" s="16"/>
+      <c r="A25" s="18"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="18"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="18"/>
+      <c r="J25" s="18"/>
     </row>
     <row r="26" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="16"/>
-      <c r="B26" s="16"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
-      <c r="G26" s="16"/>
-      <c r="H26" s="16"/>
-      <c r="I26" s="16"/>
-      <c r="J26" s="16"/>
+      <c r="A26" s="18"/>
+      <c r="B26" s="18"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="18"/>
+      <c r="I26" s="18"/>
+      <c r="J26" s="18"/>
     </row>
     <row r="27" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="16"/>
-      <c r="B27" s="16"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
-      <c r="G27" s="16"/>
-      <c r="H27" s="16"/>
-      <c r="I27" s="16"/>
-      <c r="J27" s="16"/>
+      <c r="A27" s="18"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="18"/>
+      <c r="H27" s="18"/>
+      <c r="I27" s="18"/>
+      <c r="J27" s="18"/>
     </row>
     <row r="28" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="16"/>
-      <c r="B28" s="16"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="16"/>
-      <c r="H28" s="16"/>
-      <c r="I28" s="16"/>
-      <c r="J28" s="16"/>
+      <c r="A28" s="18"/>
+      <c r="B28" s="18"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="18"/>
+      <c r="G28" s="18"/>
+      <c r="H28" s="18"/>
+      <c r="I28" s="18"/>
+      <c r="J28" s="18"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A1" location="Main!A1" display="Main" xr:uid="{62762962-8B11-4723-B541-BC1B6D5E069E}"/>
+    <hyperlink ref="C22" location="Trial!A1" display="Clinical Trials" xr:uid="{D0E1C47C-011E-4894-B1A2-4C92681F1620}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB4FECC0-655B-4808-B63E-CEE28B59A39D}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B3" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B4" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Main!A1" display="Main" xr:uid="{276F7395-BC14-456A-B952-0192CED2ACDA}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>